<commit_message>
Fix: Başak İrem Altunzincir (Başar hatası düzeltildi) + sem_generate ASCII print
- NAME_FIXES: Başar → Başak (doğru isim)
- SEM_kontrol_liste.xlsx: Başak İrem Altunzincir ve Ömer Selman Karaköse proper-case
- sem_generate.py: ✓ → OK (Windows cp1254 uyumluluğu)
- data.js/results.json yeniden üretildi

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEM_kontrol_liste.xlsx
+++ b/SEM_kontrol_liste.xlsx
@@ -3428,7 +3428,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Ömer Selman KARAKÖSE</t>
+          <t>Ömer Selman Karaköse</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Başak İrem ALTUNZİNCİR</t>
+          <t>Başak İrem Altunzincir</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">

</xml_diff>

<commit_message>
NT yarislar profilde goster; bozuk '? Serbest' satirlarini duzelt (3 sporcu)
</commit_message>
<xml_diff>
--- a/SEM_kontrol_liste.xlsx
+++ b/SEM_kontrol_liste.xlsx
@@ -48781,16 +48781,8 @@
           <t>69913227489</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>? Serbest</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>NT</t>
-        </is>
-      </c>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
           <t>100m Kelebek</t>
@@ -49047,7 +49039,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>? Serbest</t>
+          <t>1500m Serbest</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -64089,7 +64081,7 @@
       </c>
       <c r="G211" s="4" t="inlineStr">
         <is>
-          <t>? Serbest</t>
+          <t>1500m Serbest</t>
         </is>
       </c>
       <c r="H211" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Omer Selman Karakose: slot1 800m Serbest NT eklendi (yanlis silinmisti)
</commit_message>
<xml_diff>
--- a/SEM_kontrol_liste.xlsx
+++ b/SEM_kontrol_liste.xlsx
@@ -48781,8 +48781,16 @@
           <t>69913227489</t>
         </is>
       </c>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>800m Serbest</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>NT</t>
+        </is>
+      </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
           <t>100m Kelebek</t>

</xml_diff>

<commit_message>
3 yeni sporcu eklendi (TYF start listesinde olan ama Excel'de olmayan)
- Ceren TUNCAY (Kayseri, YB=12): 100m Serbest/Kurbağalama/50m Serbest
- Öykü AKÇORA (İstanbul, YB=10): 100m Serbest/Sırtüstü/100m Sırtüstü
- Sarp Barkın HASAY (İstanbul, YB=10): 100m Kelebek/Sırtüstü/200m/100m Sırtüstü

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEM_kontrol_liste.xlsx
+++ b/SEM_kontrol_liste.xlsx
@@ -45579,7 +45579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T350"/>
+  <dimension ref="A1:T353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -76415,6 +76415,223 @@
         <v/>
       </c>
     </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>350</v>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Kayseri</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Bayan</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Ceren TUNCAY</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr"/>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>100m Serbest</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>1:03.29</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>100m Kurbağalama</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>1:21.82</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>50m Serbest</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>28.72</t>
+        </is>
+      </c>
+      <c r="Q351" t="inlineStr">
+        <is>
+          <t>Kayseri</t>
+        </is>
+      </c>
+      <c r="R351">
+        <f>Q351=B351</f>
+        <v/>
+      </c>
+      <c r="T351">
+        <f>MATCH(D351,[1]Manual!$A:$A,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>351</v>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Bayan</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Öykü AKÇORA</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr"/>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>100m Serbest</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>59.19</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>50m Sırtüstü</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>30.88</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>100m Sırtüstü</t>
+        </is>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>1:05.40</t>
+        </is>
+      </c>
+      <c r="Q352" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="R352">
+        <f>Q352=B352</f>
+        <v/>
+      </c>
+      <c r="T352">
+        <f>MATCH(D352,[1]Manual!$A:$A,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Erkek</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Sarp Barkın HASAY</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr"/>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>100m Kelebek</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>57.09</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>50m Sırtüstü</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>26.85</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>200m Sırtüstü</t>
+        </is>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>2:05.72</t>
+        </is>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>100m Sırtüstü</t>
+        </is>
+      </c>
+      <c r="N353" t="inlineStr">
+        <is>
+          <t>57.28</t>
+        </is>
+      </c>
+      <c r="Q353" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="R353">
+        <f>Q353=B353</f>
+        <v/>
+      </c>
+      <c r="T353">
+        <f>MATCH(D353,[1]Manual!$A:$A,0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
46 sporcunun SEM şehri düzeltildi (kulüp şehri → SEM kayıt şehri)
Federasyon start listesi esas alındı. 43 sporcu İstanbul'dan
gerçek SEM şehirlerine taşındı (İzmir, Antalya, Ankara, Samsun vb.).
Şehir sıralaması doğru SEM bazına oturtuldu.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEM_kontrol_liste.xlsx
+++ b/SEM_kontrol_liste.xlsx
@@ -57742,7 +57742,7 @@
       </c>
       <c r="B139" s="8" t="inlineStr">
         <is>
-          <t>Eskişehir</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
@@ -59332,7 +59332,7 @@
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C157" s="5" t="inlineStr">
@@ -59402,7 +59402,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R157">
@@ -59420,7 +59420,7 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
@@ -59490,7 +59490,7 @@
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="R158">
@@ -59508,7 +59508,7 @@
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C159" s="5" t="inlineStr">
@@ -59578,7 +59578,7 @@
       </c>
       <c r="Q159" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R159">
@@ -59596,7 +59596,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
@@ -59666,7 +59666,7 @@
       </c>
       <c r="Q160" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R160">
@@ -59684,7 +59684,7 @@
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Kayseri</t>
         </is>
       </c>
       <c r="C161" s="5" t="inlineStr">
@@ -59754,7 +59754,7 @@
       </c>
       <c r="Q161" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Kayseri</t>
         </is>
       </c>
       <c r="R161">
@@ -59860,7 +59860,7 @@
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C163" s="5" t="inlineStr">
@@ -59930,7 +59930,7 @@
       </c>
       <c r="Q163" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R163">
@@ -59948,7 +59948,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
@@ -60018,7 +60018,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R164">
@@ -60036,7 +60036,7 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C165" s="5" t="inlineStr">
@@ -60106,7 +60106,7 @@
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R165">
@@ -60124,7 +60124,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Kayseri</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -60194,7 +60194,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Kayseri</t>
         </is>
       </c>
       <c r="R166">
@@ -60212,7 +60212,7 @@
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Tekirdağ</t>
         </is>
       </c>
       <c r="C167" s="5" t="inlineStr">
@@ -60274,7 +60274,7 @@
       </c>
       <c r="Q167" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Tekirdağ</t>
         </is>
       </c>
       <c r="R167">
@@ -60292,7 +60292,7 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
@@ -60362,7 +60362,7 @@
       </c>
       <c r="Q168" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R168">
@@ -60464,7 +60464,7 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
@@ -60534,7 +60534,7 @@
       </c>
       <c r="Q170" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R170">
@@ -60552,7 +60552,7 @@
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="C171" s="5" t="inlineStr">
@@ -60622,7 +60622,7 @@
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="R171">
@@ -60640,7 +60640,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Sakarya</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
@@ -60710,7 +60710,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Sakarya</t>
         </is>
       </c>
       <c r="R172">
@@ -60728,7 +60728,7 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C173" s="5" t="inlineStr">
@@ -60798,7 +60798,7 @@
       </c>
       <c r="Q173" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R173">
@@ -60816,7 +60816,7 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
@@ -60886,7 +60886,7 @@
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="R174">
@@ -60992,7 +60992,7 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
@@ -61062,7 +61062,7 @@
       </c>
       <c r="Q176" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="R176">
@@ -61080,7 +61080,7 @@
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C177" s="5" t="inlineStr">
@@ -61150,7 +61150,7 @@
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R177">
@@ -61168,7 +61168,7 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
@@ -61238,7 +61238,7 @@
       </c>
       <c r="Q178" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R178">
@@ -61256,7 +61256,7 @@
       </c>
       <c r="B179" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C179" s="5" t="inlineStr">
@@ -61326,7 +61326,7 @@
       </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R179">
@@ -61344,7 +61344,7 @@
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
@@ -61414,7 +61414,7 @@
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="R180">
@@ -61432,7 +61432,7 @@
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Gaziantep</t>
         </is>
       </c>
       <c r="C181" s="5" t="inlineStr">
@@ -61502,7 +61502,7 @@
       </c>
       <c r="Q181" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Gaziantep</t>
         </is>
       </c>
       <c r="R181">
@@ -61520,7 +61520,7 @@
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
@@ -61590,7 +61590,7 @@
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="R182">
@@ -61608,7 +61608,7 @@
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C183" s="5" t="inlineStr">
@@ -61678,7 +61678,7 @@
       </c>
       <c r="Q183" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R183">
@@ -61696,7 +61696,7 @@
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
@@ -61766,7 +61766,7 @@
       </c>
       <c r="Q184" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R184">
@@ -61784,7 +61784,7 @@
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C185" s="5" t="inlineStr">
@@ -61854,7 +61854,7 @@
       </c>
       <c r="Q185" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R185">
@@ -61872,7 +61872,7 @@
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Gaziantep</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
@@ -61942,7 +61942,7 @@
       </c>
       <c r="Q186" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Gaziantep</t>
         </is>
       </c>
       <c r="R186">
@@ -62048,7 +62048,7 @@
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Tekirdağ</t>
         </is>
       </c>
       <c r="C188" s="3" t="inlineStr">
@@ -62114,7 +62114,7 @@
       </c>
       <c r="Q188" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Tekirdağ</t>
         </is>
       </c>
       <c r="R188">
@@ -62132,7 +62132,7 @@
       </c>
       <c r="B189" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="C189" s="5" t="inlineStr">
@@ -62202,7 +62202,7 @@
       </c>
       <c r="Q189" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="R189">
@@ -62220,7 +62220,7 @@
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
@@ -62290,7 +62290,7 @@
       </c>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="R190">
@@ -62308,7 +62308,7 @@
       </c>
       <c r="B191" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C191" s="5" t="inlineStr">
@@ -62378,7 +62378,7 @@
       </c>
       <c r="Q191" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R191">
@@ -62396,7 +62396,7 @@
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
@@ -62462,7 +62462,7 @@
       </c>
       <c r="Q192" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R192">
@@ -62480,7 +62480,7 @@
       </c>
       <c r="B193" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="C193" s="5" t="inlineStr">
@@ -62550,7 +62550,7 @@
       </c>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Ankara</t>
         </is>
       </c>
       <c r="R193">
@@ -62568,7 +62568,7 @@
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
@@ -62638,7 +62638,7 @@
       </c>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R194">
@@ -62656,7 +62656,7 @@
       </c>
       <c r="B195" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Trabzon</t>
         </is>
       </c>
       <c r="C195" s="5" t="inlineStr">
@@ -62726,7 +62726,7 @@
       </c>
       <c r="Q195" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Trabzon</t>
         </is>
       </c>
       <c r="R195">
@@ -62744,7 +62744,7 @@
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
@@ -62814,7 +62814,7 @@
       </c>
       <c r="Q196" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="R196">
@@ -62920,7 +62920,7 @@
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
@@ -62990,7 +62990,7 @@
       </c>
       <c r="Q198" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R198">
@@ -63008,7 +63008,7 @@
       </c>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="C199" s="5" t="inlineStr">
@@ -63078,7 +63078,7 @@
       </c>
       <c r="Q199" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Samsun</t>
         </is>
       </c>
       <c r="R199">
@@ -63096,7 +63096,7 @@
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
@@ -63166,7 +63166,7 @@
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R200">
@@ -63184,7 +63184,7 @@
       </c>
       <c r="B201" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Sakarya</t>
         </is>
       </c>
       <c r="C201" s="5" t="inlineStr">
@@ -63254,7 +63254,7 @@
       </c>
       <c r="Q201" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Sakarya</t>
         </is>
       </c>
       <c r="R201">
@@ -63272,7 +63272,7 @@
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Bursa</t>
         </is>
       </c>
       <c r="C202" s="3" t="inlineStr">
@@ -63342,7 +63342,7 @@
       </c>
       <c r="Q202" s="6" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Bursa</t>
         </is>
       </c>
       <c r="R202">
@@ -63360,7 +63360,7 @@
       </c>
       <c r="B203" s="4" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="C203" s="5" t="inlineStr">
@@ -63430,7 +63430,7 @@
       </c>
       <c r="Q203" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>İzmir</t>
         </is>
       </c>
       <c r="R203">
@@ -63448,7 +63448,7 @@
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="C204" s="3" t="inlineStr">
@@ -63518,7 +63518,7 @@
       </c>
       <c r="Q204" t="inlineStr">
         <is>
-          <t>İstanbul</t>
+          <t>Antalya</t>
         </is>
       </c>
       <c r="R204">
@@ -64685,7 +64685,7 @@
       </c>
       <c r="B218" s="8" t="inlineStr">
         <is>
-          <t>İzmir</t>
+          <t>Trabzon</t>
         </is>
       </c>
       <c r="C218" s="3" t="inlineStr">
@@ -68305,7 +68305,7 @@
       </c>
       <c r="B259" s="8" t="inlineStr">
         <is>
-          <t>Kütahya</t>
+          <t>Eskişehir</t>
         </is>
       </c>
       <c r="C259" s="5" t="inlineStr">
@@ -76439,7 +76439,6 @@
           <t>12</t>
         </is>
       </c>
-      <c r="F351" t="inlineStr"/>
       <c r="G351" t="inlineStr">
         <is>
           <t>100m Serbest</t>
@@ -76468,6 +76467,11 @@
       <c r="L351" t="inlineStr">
         <is>
           <t>28.72</t>
+        </is>
+      </c>
+      <c r="P351" t="inlineStr">
+        <is>
+          <t>Kayseri Su Sporları Spor Kulübü</t>
         </is>
       </c>
       <c r="Q351" t="inlineStr">
@@ -76508,7 +76512,6 @@
           <t>10</t>
         </is>
       </c>
-      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>100m Serbest</t>
@@ -76537,6 +76540,11 @@
       <c r="L352" t="inlineStr">
         <is>
           <t>1:05.40</t>
+        </is>
+      </c>
+      <c r="P352" t="inlineStr">
+        <is>
+          <t>Enka Spor Kulübü</t>
         </is>
       </c>
       <c r="Q352" t="inlineStr">
@@ -76577,7 +76585,6 @@
           <t>10</t>
         </is>
       </c>
-      <c r="F353" t="inlineStr"/>
       <c r="G353" t="inlineStr">
         <is>
           <t>100m Kelebek</t>
@@ -76616,6 +76623,11 @@
       <c r="N353" t="inlineStr">
         <is>
           <t>57.28</t>
+        </is>
+      </c>
+      <c r="P353" t="inlineStr">
+        <is>
+          <t>Enka Spor Kulübü</t>
         </is>
       </c>
       <c r="Q353" t="inlineStr">

</xml_diff>

<commit_message>
Sureleri guncelle: 56 sure TYF/manuel duzeltme uygulandı (backup oncesi) Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEM_kontrol_liste.xlsx
+++ b/SEM_kontrol_liste.xlsx
@@ -59714,7 +59714,7 @@
       </c>
       <c r="H161" s="4" t="inlineStr">
         <is>
-          <t>2:24.85</t>
+          <t>2:18.03</t>
         </is>
       </c>
       <c r="I161" s="4" t="inlineStr">
@@ -60876,7 +60876,7 @@
       </c>
       <c r="N174" s="4" t="inlineStr">
         <is>
-          <t>3:11.89</t>
+          <t>3:07.35</t>
         </is>
       </c>
       <c r="P174" t="inlineStr">
@@ -61996,7 +61996,7 @@
       </c>
       <c r="J187" s="4" t="inlineStr">
         <is>
-          <t>2:44.64</t>
+          <t>2:40.28</t>
         </is>
       </c>
       <c r="K187" s="4" t="inlineStr">
@@ -62256,7 +62256,7 @@
       </c>
       <c r="J190" s="2" t="inlineStr">
         <is>
-          <t>30.79</t>
+          <t>30.25</t>
         </is>
       </c>
       <c r="K190" s="2" t="inlineStr">
@@ -62276,7 +62276,7 @@
       </c>
       <c r="N190" s="2" t="inlineStr">
         <is>
-          <t>1:54.46</t>
+          <t>1:08.78</t>
         </is>
       </c>
       <c r="P190" t="inlineStr">
@@ -62716,7 +62716,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>5:35.19</t>
         </is>
       </c>
       <c r="P195" t="inlineStr">
@@ -62950,7 +62950,7 @@
       </c>
       <c r="H198" s="4" t="inlineStr">
         <is>
-          <t>1:03.10</t>
+          <t>1:02.32</t>
         </is>
       </c>
       <c r="I198" s="4" t="inlineStr">
@@ -62960,7 +62960,7 @@
       </c>
       <c r="J198" s="4" t="inlineStr">
         <is>
-          <t>1:13.14</t>
+          <t>1:12.45</t>
         </is>
       </c>
       <c r="K198" s="4" t="inlineStr">
@@ -62970,7 +62970,7 @@
       </c>
       <c r="L198" s="4" t="inlineStr">
         <is>
-          <t>2:18.60</t>
+          <t>2:16.56</t>
         </is>
       </c>
       <c r="M198" s="4" t="inlineStr">
@@ -62980,7 +62980,7 @@
       </c>
       <c r="N198" s="4" t="inlineStr">
         <is>
-          <t>2:48.20</t>
+          <t>2:35.67</t>
         </is>
       </c>
       <c r="P198" t="inlineStr">
@@ -63126,7 +63126,7 @@
       </c>
       <c r="H200" s="4" t="inlineStr">
         <is>
-          <t>27.67</t>
+          <t>26.88</t>
         </is>
       </c>
       <c r="I200" s="4" t="inlineStr">
@@ -63234,7 +63234,7 @@
       </c>
       <c r="L201" s="2" t="inlineStr">
         <is>
-          <t>1:10.35</t>
+          <t>1:07.61</t>
         </is>
       </c>
       <c r="M201" s="2" t="inlineStr">
@@ -63302,7 +63302,7 @@
       </c>
       <c r="H202" s="4" t="inlineStr">
         <is>
-          <t>1:18.34</t>
+          <t>1:15.64</t>
         </is>
       </c>
       <c r="I202" s="4" t="inlineStr">
@@ -63332,7 +63332,7 @@
       </c>
       <c r="N202" s="4" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>5:49.65</t>
         </is>
       </c>
       <c r="P202" s="12" t="inlineStr">
@@ -63410,7 +63410,7 @@
       </c>
       <c r="L203" s="2" t="inlineStr">
         <is>
-          <t>4:13.50</t>
+          <t>4:06.09</t>
         </is>
       </c>
       <c r="M203" s="2" t="inlineStr">
@@ -63498,7 +63498,7 @@
       </c>
       <c r="L204" s="4" t="inlineStr">
         <is>
-          <t>10:58.63</t>
+          <t>10:42.33</t>
         </is>
       </c>
       <c r="M204" s="4" t="inlineStr">
@@ -63508,7 +63508,7 @@
       </c>
       <c r="N204" s="4" t="inlineStr">
         <is>
-          <t>2:50.01</t>
+          <t>2:47.79</t>
         </is>
       </c>
       <c r="P204" t="inlineStr">
@@ -63576,7 +63576,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>2:42.01</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr">
@@ -63596,7 +63596,7 @@
       </c>
       <c r="N205" s="2" t="inlineStr">
         <is>
-          <t>2:50.30</t>
+          <t>2:45.93</t>
         </is>
       </c>
       <c r="P205" t="inlineStr">
@@ -63654,7 +63654,7 @@
       </c>
       <c r="H206" s="4" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>19:52.42</t>
         </is>
       </c>
       <c r="I206" s="4" t="inlineStr">
@@ -63684,7 +63684,7 @@
       </c>
       <c r="N206" s="4" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>6:01.82</t>
         </is>
       </c>
       <c r="P206" s="12" t="inlineStr">
@@ -63742,7 +63742,7 @@
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
-          <t>10:37.45</t>
+          <t>9:42.66</t>
         </is>
       </c>
       <c r="I207" s="2" t="inlineStr">
@@ -63752,7 +63752,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2:53.05</t>
+          <t>2:38.68</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -63762,7 +63762,7 @@
       </c>
       <c r="L207" s="2" t="inlineStr">
         <is>
-          <t>21:34.28</t>
+          <t>18:34.24</t>
         </is>
       </c>
       <c r="M207" s="2" t="inlineStr">
@@ -63772,7 +63772,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>5:51.23</t>
+          <t>5:30.64</t>
         </is>
       </c>
       <c r="P207" t="inlineStr">
@@ -63835,7 +63835,7 @@
       </c>
       <c r="H208" s="4" t="inlineStr">
         <is>
-          <t>1:02.12</t>
+          <t>1:00.44</t>
         </is>
       </c>
       <c r="I208" s="4" t="inlineStr">
@@ -63855,7 +63855,7 @@
       </c>
       <c r="L208" s="4" t="inlineStr">
         <is>
-          <t>1:04.67</t>
+          <t>1:03.62</t>
         </is>
       </c>
       <c r="M208" s="4" t="inlineStr">
@@ -63865,7 +63865,7 @@
       </c>
       <c r="N208" s="4" t="inlineStr">
         <is>
-          <t>2:35.32</t>
+          <t>2:26.78</t>
         </is>
       </c>
       <c r="P208" t="inlineStr">
@@ -63933,7 +63933,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>3:00.11</t>
+          <t>2:36.07</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -63953,7 +63953,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>2:55.74</t>
+          <t>2:34.89</t>
         </is>
       </c>
       <c r="P209" t="inlineStr">
@@ -64207,7 +64207,7 @@
       </c>
       <c r="L212" s="4" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>8:46.58</t>
         </is>
       </c>
       <c r="M212" s="4" t="inlineStr">
@@ -64466,7 +64466,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>23:14.93</t>
+          <t>20:10.47</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr">
@@ -64476,7 +64476,7 @@
       </c>
       <c r="L215" s="2" t="inlineStr">
         <is>
-          <t>12:01.37</t>
+          <t>10:27.69</t>
         </is>
       </c>
       <c r="M215" s="2" t="inlineStr">
@@ -64486,7 +64486,7 @@
       </c>
       <c r="N215" s="2" t="inlineStr">
         <is>
-          <t>2:45.97</t>
+          <t>2:39.60</t>
         </is>
       </c>
       <c r="P215" t="inlineStr">
@@ -64544,7 +64544,7 @@
       </c>
       <c r="H216" s="4" t="inlineStr">
         <is>
-          <t>34.96</t>
+          <t>33.88</t>
         </is>
       </c>
       <c r="I216" s="4" t="inlineStr">
@@ -64554,7 +64554,7 @@
       </c>
       <c r="J216" s="4" t="inlineStr">
         <is>
-          <t>1:05.17</t>
+          <t>1:04.61</t>
         </is>
       </c>
       <c r="K216" s="4" t="inlineStr">
@@ -64564,7 +64564,7 @@
       </c>
       <c r="L216" s="4" t="inlineStr">
         <is>
-          <t>1:18.39</t>
+          <t>1:14.50</t>
         </is>
       </c>
       <c r="M216" s="4" t="inlineStr">
@@ -64574,7 +64574,7 @@
       </c>
       <c r="N216" s="4" t="inlineStr">
         <is>
-          <t>2:27.96</t>
+          <t>2:26.64</t>
         </is>
       </c>
       <c r="P216" t="inlineStr">
@@ -64818,7 +64818,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>31.58</t>
+          <t>30.95</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -65366,7 +65366,7 @@
       </c>
       <c r="L225" s="2" t="inlineStr">
         <is>
-          <t>1:17.94</t>
+          <t>1:16.05</t>
         </is>
       </c>
       <c r="M225" s="2" t="inlineStr">
@@ -65376,7 +65376,7 @@
       </c>
       <c r="N225" s="2" t="inlineStr">
         <is>
-          <t>6:23.01</t>
+          <t>6:09.57</t>
         </is>
       </c>
       <c r="P225" t="inlineStr">
@@ -65434,7 +65434,7 @@
       </c>
       <c r="H226" s="4" t="inlineStr">
         <is>
-          <t>11:48.36</t>
+          <t>10:45.92</t>
         </is>
       </c>
       <c r="I226" s="4" t="inlineStr">
@@ -65444,7 +65444,7 @@
       </c>
       <c r="J226" s="4" t="inlineStr">
         <is>
-          <t>2:46.48</t>
+          <t>2:44.17</t>
         </is>
       </c>
       <c r="K226" s="4" t="inlineStr">
@@ -65464,7 +65464,7 @@
       </c>
       <c r="N226" s="4" t="inlineStr">
         <is>
-          <t>2:50.65</t>
+          <t>2:49.61</t>
         </is>
       </c>
       <c r="P226" t="inlineStr">
@@ -65874,7 +65874,7 @@
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
-          <t>11:43.65</t>
+          <t>10:29.68</t>
         </is>
       </c>
       <c r="I231" s="2" t="inlineStr">
@@ -65894,7 +65894,7 @@
       </c>
       <c r="L231" s="2" t="inlineStr">
         <is>
-          <t>22:49.37</t>
+          <t>20:03.79</t>
         </is>
       </c>
       <c r="M231" s="2" t="inlineStr">
@@ -65904,7 +65904,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>5:45.97</t>
         </is>
       </c>
       <c r="P231" s="12" t="inlineStr">
@@ -74178,7 +74178,7 @@
       </c>
       <c r="L325" s="4" t="inlineStr">
         <is>
-          <t>1:15.34</t>
+          <t>1:13.94</t>
         </is>
       </c>
       <c r="M325" s="4" t="inlineStr">
@@ -74188,7 +74188,7 @@
       </c>
       <c r="N325" s="4" t="inlineStr">
         <is>
-          <t>2:49.58</t>
+          <t>2:47.58</t>
         </is>
       </c>
       <c r="P325" t="inlineStr">
@@ -74246,7 +74246,7 @@
       </c>
       <c r="H326" s="2" t="inlineStr">
         <is>
-          <t>1:04.08</t>
+          <t>1:03.14</t>
         </is>
       </c>
       <c r="I326" s="2" t="inlineStr">
@@ -74256,7 +74256,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>1:13.80</t>
+          <t>1:11.62</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr">
@@ -74344,7 +74344,7 @@
       </c>
       <c r="J327" s="4" t="inlineStr">
         <is>
-          <t>2:46.50</t>
+          <t>2:41.55</t>
         </is>
       </c>
       <c r="K327" s="4" t="inlineStr">
@@ -74442,7 +74442,7 @@
       </c>
       <c r="L328" s="2" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>1:29.53</t>
         </is>
       </c>
       <c r="M328" s="2" t="inlineStr">
@@ -74540,7 +74540,7 @@
       </c>
       <c r="N329" s="4" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>5:52.17</t>
         </is>
       </c>
       <c r="P329" t="inlineStr">
@@ -74706,7 +74706,7 @@
       </c>
       <c r="L331" s="4" t="inlineStr">
         <is>
-          <t>1:13.51</t>
+          <t>1:12.64</t>
         </is>
       </c>
       <c r="M331" s="4" t="inlineStr">
@@ -74784,7 +74784,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>10:22.10</t>
+          <t>10:12.52</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Yarisan oncesi son guncelleme: DNS mantigi + 8 sure duzeltme + panel iyilestirme Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEM_kontrol_liste.xlsx
+++ b/SEM_kontrol_liste.xlsx
@@ -62540,7 +62540,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>30.40</t>
+          <t>30.33</t>
         </is>
       </c>
       <c r="P193" t="inlineStr">
@@ -63214,7 +63214,7 @@
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
-          <t>31.99</t>
+          <t>31.60</t>
         </is>
       </c>
       <c r="I201" s="2" t="inlineStr">
@@ -64099,7 +64099,7 @@
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
-          <t>26.53</t>
+          <t>26.45</t>
         </is>
       </c>
       <c r="I211" s="2" t="inlineStr">
@@ -64378,7 +64378,7 @@
       </c>
       <c r="J214" s="4" t="inlineStr">
         <is>
-          <t>1:08.66</t>
+          <t>1:08.49</t>
         </is>
       </c>
       <c r="K214" s="4" t="inlineStr">
@@ -65097,7 +65097,7 @@
       </c>
       <c r="L222" s="4" t="inlineStr">
         <is>
-          <t>1:29.67</t>
+          <t>1:27.38</t>
         </is>
       </c>
       <c r="M222" s="4" t="inlineStr">
@@ -74158,7 +74158,7 @@
       </c>
       <c r="H325" s="4" t="inlineStr">
         <is>
-          <t>1:08.52</t>
+          <t>1:08.45</t>
         </is>
       </c>
       <c r="I325" s="4" t="inlineStr">
@@ -74520,7 +74520,7 @@
       </c>
       <c r="J329" s="4" t="inlineStr">
         <is>
-          <t>2:43.29</t>
+          <t>2:42.84</t>
         </is>
       </c>
       <c r="K329" s="4" t="inlineStr">
@@ -74804,7 +74804,7 @@
       </c>
       <c r="N332" s="2" t="inlineStr">
         <is>
-          <t>19:45.31</t>
+          <t>19:45.16</t>
         </is>
       </c>
       <c r="P332" s="6" t="inlineStr">

</xml_diff>